<commit_message>
Add more entries based on gameplay testing; modified some voice_name coding for creatures that I've made specific sfx for (e.g., mountain_giant, elementals, etc.)
</commit_message>
<xml_diff>
--- a/corrections/new_entries.xlsx
+++ b/corrections/new_entries.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\Desktop\wow_vo_webui\corrections\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31DE981F-6BA6-427F-B9F1-22622FA208D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{09166896-9492-416B-A320-56FC30FD87A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4121" uniqueCount="1096">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4151" uniqueCount="1106">
   <si>
     <t>source</t>
   </si>
@@ -3493,6 +3493,36 @@
   </si>
   <si>
     <t>Kravel Koalbeard</t>
+  </si>
+  <si>
+    <t>Bat Handler Camille</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You seek passage somewhere, adventurer? My bats will get you there in no time. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">You're going to pull off a stunt on Jack in front of his boys? That takes a good amount of; stupidity. Well, it's going to cost you. I'm not going to risk my life for anything less than a gold. And you best wait til I'm out of the way before you make a move. </t>
+  </si>
+  <si>
+    <t>Olga, the Scalawag Wench</t>
+  </si>
+  <si>
+    <t>Annie Bonn</t>
+  </si>
+  <si>
+    <t>That cursed Jonah Sterling will lead us right into doom. If he spent more time outside of his cave, he would realize the folly of attacking professional navies in a time of war.</t>
+  </si>
+  <si>
+    <t>Old Icefin draws in the sand. From the crude pictures he traces you can make out that he wants your help.</t>
+  </si>
+  <si>
+    <t>Old Icefin</t>
+  </si>
+  <si>
+    <t>Are you ready to begin the assault and win back the Undercity for the Horde, adventurer?</t>
+  </si>
+  <si>
+    <t>The elements are with us in force, adventurer; with their help, we will do  all that is in our power to stop Varimathras and Putress! Loktaro garr!</t>
   </si>
 </sst>
 </file>
@@ -3828,7 +3858,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K706"/>
+  <dimension ref="A1:K712"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="7" max="7" width="17.7109375" customWidth="1"/>
@@ -27822,6 +27852,180 @@
       </c>
       <c r="K706">
         <v>-88</v>
+      </c>
+    </row>
+    <row r="707" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A707" t="s">
+        <v>205</v>
+      </c>
+      <c r="D707" t="s">
+        <v>1097</v>
+      </c>
+      <c r="E707">
+        <v>5</v>
+      </c>
+      <c r="F707">
+        <v>1</v>
+      </c>
+      <c r="G707" t="s">
+        <v>1096</v>
+      </c>
+      <c r="H707" t="s">
+        <v>12</v>
+      </c>
+      <c r="I707">
+        <v>23816</v>
+      </c>
+      <c r="J707" t="s">
+        <v>1097</v>
+      </c>
+      <c r="K707">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="708" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A708" t="s">
+        <v>205</v>
+      </c>
+      <c r="D708" t="s">
+        <v>1098</v>
+      </c>
+      <c r="E708">
+        <v>-77</v>
+      </c>
+      <c r="F708">
+        <v>-77</v>
+      </c>
+      <c r="G708" t="s">
+        <v>1099</v>
+      </c>
+      <c r="H708" t="s">
+        <v>12</v>
+      </c>
+      <c r="I708">
+        <v>24639</v>
+      </c>
+      <c r="J708" t="s">
+        <v>1098</v>
+      </c>
+      <c r="K708">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="709" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A709" t="s">
+        <v>205</v>
+      </c>
+      <c r="D709" t="s">
+        <v>1101</v>
+      </c>
+      <c r="E709">
+        <v>1</v>
+      </c>
+      <c r="F709">
+        <v>1</v>
+      </c>
+      <c r="G709" t="s">
+        <v>1100</v>
+      </c>
+      <c r="H709" t="s">
+        <v>12</v>
+      </c>
+      <c r="I709">
+        <v>24741</v>
+      </c>
+      <c r="J709" t="s">
+        <v>1101</v>
+      </c>
+      <c r="K709">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="710" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A710" t="s">
+        <v>205</v>
+      </c>
+      <c r="D710" t="s">
+        <v>1102</v>
+      </c>
+      <c r="E710">
+        <v>-77</v>
+      </c>
+      <c r="F710">
+        <v>-77</v>
+      </c>
+      <c r="G710" t="s">
+        <v>1103</v>
+      </c>
+      <c r="H710" t="s">
+        <v>12</v>
+      </c>
+      <c r="I710">
+        <v>24544</v>
+      </c>
+      <c r="J710" t="s">
+        <v>1102</v>
+      </c>
+      <c r="K710">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="711" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A711" t="s">
+        <v>205</v>
+      </c>
+      <c r="D711" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E711">
+        <v>2</v>
+      </c>
+      <c r="F711">
+        <v>0</v>
+      </c>
+      <c r="G711" t="s">
+        <v>358</v>
+      </c>
+      <c r="H711" t="s">
+        <v>12</v>
+      </c>
+      <c r="I711">
+        <v>31650</v>
+      </c>
+      <c r="J711" t="s">
+        <v>1104</v>
+      </c>
+      <c r="K711">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="712" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A712" t="s">
+        <v>205</v>
+      </c>
+      <c r="D712" t="s">
+        <v>1105</v>
+      </c>
+      <c r="E712">
+        <v>2</v>
+      </c>
+      <c r="F712">
+        <v>0</v>
+      </c>
+      <c r="G712" t="s">
+        <v>358</v>
+      </c>
+      <c r="H712" t="s">
+        <v>12</v>
+      </c>
+      <c r="I712">
+        <v>31650</v>
+      </c>
+      <c r="J712" t="s">
+        <v>1105</v>
+      </c>
+      <c r="K712">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>